<commit_message>
added the remaining card combinations and stored them in script
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f734f07fa70639b/Documents/GitHub/CS425-426/Assets/StreamingAssets/Excel/Value/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{F7CA5EFD-5273-4130-AB32-818DA4AAA797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C398C3F-870D-4889-BDB3-9FD9A98C6C4E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CED1D2B-BC80-4E66-98DC-CE76671592DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1224" yWindow="4308" windowWidth="19404" windowHeight="9372" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="101">
   <si>
     <t>ID</t>
   </si>
@@ -302,6 +302,57 @@
   </si>
   <si>
     <t>Becomes alert and sidesteps. Evades 100% the next incoming hit.</t>
+  </si>
+  <si>
+    <t>Overdrive Dose</t>
+  </si>
+  <si>
+    <t>Combat Stimulant</t>
+  </si>
+  <si>
+    <t>Balanced Formula</t>
+  </si>
+  <si>
+    <t>Rebirth Capsule</t>
+  </si>
+  <si>
+    <t>Titan Formula</t>
+  </si>
+  <si>
+    <t>Battle Brew</t>
+  </si>
+  <si>
+    <t>Adrenal Surge</t>
+  </si>
+  <si>
+    <t>Berserker Serum</t>
+  </si>
+  <si>
+    <t>Fury Rebirth</t>
+  </si>
+  <si>
+    <t>Aggression Compound</t>
+  </si>
+  <si>
+    <t>Drunken Rage</t>
+  </si>
+  <si>
+    <t>Adrenal Mix</t>
+  </si>
+  <si>
+    <t>Reflex Booster</t>
+  </si>
+  <si>
+    <t>Bio-Regen Formula</t>
+  </si>
+  <si>
+    <t>Nerve Enhancer</t>
+  </si>
+  <si>
+    <t>Survivor's Brew</t>
+  </si>
+  <si>
+    <t>Soul Brew</t>
   </si>
 </sst>
 </file>
@@ -619,17 +670,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G46"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="24.88671875" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" customWidth="1"/>
-    <col min="6" max="6" width="101.6640625" customWidth="1"/>
-    <col min="7" max="7" width="121.44140625" customWidth="1"/>
+    <col min="2" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="101.7109375" customWidth="1"/>
+    <col min="7" max="7" width="121.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -652,7 +703,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>ROW()-2</f>
         <v>0</v>
@@ -676,7 +727,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" ref="A3:A21" si="0">ROW()-2</f>
         <v>1</v>
@@ -700,7 +751,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -724,7 +775,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -748,7 +799,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -772,7 +823,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -796,7 +847,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -820,7 +871,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -844,7 +895,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -868,7 +919,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -892,7 +943,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -916,7 +967,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -940,7 +991,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -964,7 +1015,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -988,7 +1039,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1012,7 +1063,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1036,7 +1087,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1060,7 +1111,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1084,7 +1135,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1108,7 +1159,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1132,171 +1183,477 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
-        <f t="shared" ref="A22:A29" si="1">ROW()-2</f>
+        <f>ROW()-2</f>
         <v>20</v>
       </c>
       <c r="B22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <f>ROW()-2</f>
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <f>ROW()-2</f>
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <f>ROW()-2</f>
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <f>ROW()-2</f>
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <f>ROW()-2</f>
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <f>ROW()-2</f>
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <f>ROW()-2</f>
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <f>ROW()-2</f>
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>92</v>
+      </c>
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <f>ROW()-2</f>
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <f>ROW()-2</f>
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
+        <v>94</v>
+      </c>
+      <c r="C32" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <f>ROW()-2</f>
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <f>ROW()-2</f>
+        <v>32</v>
+      </c>
+      <c r="B34" t="s">
+        <v>96</v>
+      </c>
+      <c r="C34" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <f>ROW()-2</f>
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <f>ROW()-2</f>
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
+        <v>98</v>
+      </c>
+      <c r="C36" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <f>ROW()-2</f>
+        <v>35</v>
+      </c>
+      <c r="B37" t="s">
+        <v>99</v>
+      </c>
+      <c r="C37" t="s">
+        <v>6</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <f>ROW()-2</f>
+        <v>36</v>
+      </c>
+      <c r="B38" t="s">
+        <v>100</v>
+      </c>
+      <c r="C38" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <f t="shared" ref="A39:A45" si="1">ROW()-2</f>
+        <v>37</v>
+      </c>
+      <c r="B39" t="s">
         <v>71</v>
       </c>
-      <c r="C22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22" t="s">
-        <v>4</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="C39" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40">
         <f t="shared" si="1"/>
-        <v>21</v>
-      </c>
-      <c r="B23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40" t="s">
         <v>70</v>
       </c>
-      <c r="C23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23" t="s">
-        <v>4</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="C40" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40" t="s">
+        <v>4</v>
+      </c>
+      <c r="F40" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41">
         <f t="shared" si="1"/>
-        <v>22</v>
-      </c>
-      <c r="B24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" t="s">
         <v>69</v>
       </c>
-      <c r="C24" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24">
-        <v>0</v>
-      </c>
-      <c r="E24" t="s">
-        <v>4</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="C41" t="s">
+        <v>6</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>4</v>
+      </c>
+      <c r="F41" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42">
         <f t="shared" si="1"/>
-        <v>23</v>
-      </c>
-      <c r="B25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" t="s">
         <v>68</v>
       </c>
-      <c r="C25" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="E25" t="s">
-        <v>4</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="C42" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>4</v>
+      </c>
+      <c r="F42" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
         <f t="shared" si="1"/>
-        <v>24</v>
-      </c>
-      <c r="B26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" t="s">
         <v>76</v>
       </c>
-      <c r="C26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26" t="s">
-        <v>4</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="C43" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43" t="s">
+        <v>4</v>
+      </c>
+      <c r="F43" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44">
         <f t="shared" si="1"/>
-        <v>25</v>
-      </c>
-      <c r="B27" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" t="s">
         <v>77</v>
       </c>
-      <c r="C27" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27">
-        <v>0</v>
-      </c>
-      <c r="E27" t="s">
-        <v>4</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="C44" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44" t="s">
+        <v>4</v>
+      </c>
+      <c r="F44" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45">
         <f t="shared" si="1"/>
-        <v>26</v>
-      </c>
-      <c r="B28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" t="s">
         <v>80</v>
       </c>
-      <c r="C28" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28">
-        <v>0</v>
-      </c>
-      <c r="E28" t="s">
-        <v>4</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="C45" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45" t="s">
+        <v>4</v>
+      </c>
+      <c r="F45" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <f t="shared" si="1"/>
-        <v>27</v>
-      </c>
-      <c r="B29" t="s">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <f>ROW()-2</f>
+        <v>44</v>
+      </c>
+      <c r="B46" t="s">
         <v>81</v>
       </c>
-      <c r="C29" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29">
-        <v>0</v>
-      </c>
-      <c r="E29" t="s">
-        <v>4</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="C46" t="s">
+        <v>6</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>4</v>
+      </c>
+      <c r="F46" t="s">
         <v>83</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated the excel for the items
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CED1D2B-BC80-4E66-98DC-CE76671592DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44221EBC-0D2F-4E3C-B3A3-065CBFA31B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="135">
   <si>
     <t>ID</t>
   </si>
@@ -229,9 +229,6 @@
     <t>Heal(percent=0.25); StopBleeding(); IncreaseAttack(percent=0.23; turns=1);</t>
   </si>
   <si>
-    <t>Heal(percent=0.25); StopBleeding(); IncreaseAttack(percent=0.25; turns=2); IncreaseDefense(percent=-0.15; turns=2); Heal(percent=-0.10);</t>
-  </si>
-  <si>
     <t>Heal(percent=0.25); StopBleeding(); IncreaseAttack(percent=0.23; turns=2); IncreaseDefense(percent=0.23; turns=2);</t>
   </si>
   <si>
@@ -353,6 +350,111 @@
   </si>
   <si>
     <t>Soul Brew</t>
+  </si>
+  <si>
+    <t>increases critical chance by (Beer % + (rarity of card)) for 3 turns and revives player to (Revival Serum % + (rarity of card))</t>
+  </si>
+  <si>
+    <t>increases critical chance by (Beer % + (rarity of card)) for 2 turns, heals (Medkit %  + (rarity of card)) and stops bleeding</t>
+  </si>
+  <si>
+    <t>increases defense and attack by (Drugs %  + (rarity of card)) and increases critical chance by (Beer % + (rarity of card)) for 2 turns</t>
+  </si>
+  <si>
+    <t>increases defense and attack by (Drugs % + (rarity of card)) for 3 turns and revives player to (Revival Serum % + (rarity of card))</t>
+  </si>
+  <si>
+    <t>increases defense and attack by (Drugs % + (rarity of card)) and increases critical damage by (Syringe % + (rarity of card)) for 2 turns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">increases defense and attack by (Drugs % + (rarity of card)) for 2 turns, heals (Medkit % + (rarity of card)) and stops bleeding </t>
+  </si>
+  <si>
+    <t>increases attack, decreases defense and health by (Rage Pill %), and increases critical chance by (Beer %) for 2 turns</t>
+  </si>
+  <si>
+    <t>increases attack by (Rage Pill % + (rarity of card)) and decreases defense and health by (Rage Pill % + Drugs % + (rarity of card)) for 2 turns</t>
+  </si>
+  <si>
+    <t>increases attack, decreases defense and health by (Rage Pill % + (rarity of card)) for 3 turns and revives player to (Revival Serum % + (rarity of card))</t>
+  </si>
+  <si>
+    <t>heals (Medkit % + (rarity of card)), stops bleeding increases attack, decreases defense and health by (Rage Pill % + (rarity of card)) for 1 turns</t>
+  </si>
+  <si>
+    <t>increases attack, lowers defense and health by (Rage Pill % + (rarity of card)) and increases critical damage by (Syringe % + (rarity of card)) for 2 turns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">increases attack by (Pills % + (rarity of card)) and critical chance by (Beer %  + (rarity of card)) for 2 turns </t>
+  </si>
+  <si>
+    <t>increases attack by (Pills % + (rarity of card)), defense and attack by (Drugs % + (rarity of card)) for 2 turns</t>
+  </si>
+  <si>
+    <t>increases attack by (Pills % + (rarity of card)) for 3 turns and revives player to (Revival Serum % + (rarity of card))</t>
+  </si>
+  <si>
+    <t>increases attack by (Pills % + (rarity of card)) and heals (Medkit %  + (rarity of card)) for 2 turns</t>
+  </si>
+  <si>
+    <t>increases attack by (Pills % + (rarity of card)) and critical damage by (Syringe % + (rarity of card)) for 2 turns</t>
+  </si>
+  <si>
+    <t>increases attack by (Pills and Rage Pill % + (rarity of card)), lowers defense and health by (Rage Pill % + (rarity of card)) for 2 turns</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); LowerDefense(percent=0.15; turns = 2); LowerHealth(percent = 0.1; turns = 2);</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); IncreaseCritChance(percent = 0.15; turns = 2);</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.20; turns = 2); IncreaseDefense(percent = 0.15; turns = 2);</t>
+  </si>
+  <si>
+    <t>Heal(percent=0.17; turns = 2); StopBleeding(); LowerDefense(percent=0.15; turns = 2); LowerHealth(percent = 0.1; turns = 2)</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2);IncreaseCritDamage(percent = 0.2; turns = 2)</t>
+  </si>
+  <si>
+    <t>IncreaseCriticalChance(percent=0.17; turns = 2); Heal(percent = 0.25); StopBleeding();</t>
+  </si>
+  <si>
+    <t>IncreaseDefense(percent=0.17; turns = 3); IncreaseAttack(percent=0.15; turns = 3); Revive(percent = 0.3);</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); LowerDefense(percent=0.15;  turns = 2); LowerHealth(percent = 0.1; turns = 2);</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); LowerDefense(percent=0.15; turns = 2); LowerHealth(percent = 0.1; turns = 2); Revive(percent=0.2)</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); DecreaseDefense(percent=0.15; turns = 2); LowerHealth(percent = 0.2; turns = 2); IncreaseCritChance(percent=0.2; turns  = 2);</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); LowerDefense(percent=0.15; turns = 2); LowerHealth(percent = 0.1; turns = 2); IncreaseCritDamage(percent=0.15; turns = 2);</t>
+  </si>
+  <si>
+    <t>Heal(percent=0.25); StopBleeding(); IncreaseAttack(percent=0.25; turns=2); IncreaseDefense(percent=0.15; turns=2); Heal(percent=-0.10);</t>
+  </si>
+  <si>
+    <t>IncreaseDefense(percent=0.17; turns = 2); IncreaseAttack(percent=0.15; turns = 2); IncreaseCritChance(percent = 0.15; turns = 3);</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); Heal(percent = 0.25);</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); Revive(percent = 0.2)</t>
+  </si>
+  <si>
+    <t>IncreaseCriticalChance(percent=0.17; turns = 3); Revive(percent = 0.3);</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); IncreaseDefense(percent=0.17; turns = 2); IncreaseCritDamage(percent=0.15; turns = 2);</t>
+  </si>
+  <si>
+    <t>IncreaseAttack(percent=0.17; turns = 2); IncreaseDefense(percent=0.17; turns = 2); StopBleeding(); Heal(percent = 0.3);</t>
   </si>
 </sst>
 </file>
@@ -671,16 +773,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="24.85546875" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" customWidth="1"/>
-    <col min="6" max="6" width="101.7109375" customWidth="1"/>
-    <col min="7" max="7" width="121.42578125" customWidth="1"/>
+    <col min="2" max="3" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="24.88671875" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" customWidth="1"/>
+    <col min="6" max="6" width="101.6640625" customWidth="1"/>
+    <col min="7" max="7" width="121.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -700,10 +802,10 @@
         <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <f>ROW()-2</f>
         <v>0</v>
@@ -727,7 +829,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" ref="A3:A21" si="0">ROW()-2</f>
         <v>1</v>
@@ -751,7 +853,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -775,7 +877,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -799,7 +901,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -823,7 +925,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -847,7 +949,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -871,7 +973,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -895,7 +997,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -919,7 +1021,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -937,13 +1039,13 @@
         <v>4</v>
       </c>
       <c r="F11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G11" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -967,7 +1069,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -991,7 +1093,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1015,7 +1117,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1039,7 +1141,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1060,10 +1162,10 @@
         <v>43</v>
       </c>
       <c r="G16" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1084,10 +1186,10 @@
         <v>44</v>
       </c>
       <c r="G17" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1108,10 +1210,10 @@
         <v>45</v>
       </c>
       <c r="G18" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1132,10 +1234,10 @@
         <v>42</v>
       </c>
       <c r="G19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1156,10 +1258,10 @@
         <v>38</v>
       </c>
       <c r="G20" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1180,449 +1282,551 @@
         <v>40</v>
       </c>
       <c r="G21" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
-        <f>ROW()-2</f>
+        <f t="shared" ref="A22:A38" si="1">ROW()-2</f>
         <v>20</v>
       </c>
       <c r="B22" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>4</v>
+      </c>
+      <c r="F22" t="s">
+        <v>116</v>
+      </c>
+      <c r="G22" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
         <v>84</v>
       </c>
-      <c r="C22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <f>ROW()-2</f>
-        <v>21</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>4</v>
+      </c>
+      <c r="F23" t="s">
+        <v>115</v>
+      </c>
+      <c r="G23" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
         <v>85</v>
       </c>
-      <c r="C23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <f>ROW()-2</f>
-        <v>22</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" t="s">
+        <v>114</v>
+      </c>
+      <c r="G24" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
         <v>86</v>
       </c>
-      <c r="C24" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24">
-        <v>0</v>
-      </c>
-      <c r="E24" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <f>ROW()-2</f>
-        <v>23</v>
-      </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>4</v>
+      </c>
+      <c r="F25" t="s">
+        <v>113</v>
+      </c>
+      <c r="G25" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
         <v>87</v>
       </c>
-      <c r="C25" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="E25" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <f>ROW()-2</f>
-        <v>24</v>
-      </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26" t="s">
+        <v>4</v>
+      </c>
+      <c r="F26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G26" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
         <v>88</v>
       </c>
-      <c r="C26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <f>ROW()-2</f>
-        <v>25</v>
-      </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27" t="s">
+        <v>4</v>
+      </c>
+      <c r="F27" t="s">
+        <v>111</v>
+      </c>
+      <c r="G27" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
         <v>89</v>
       </c>
-      <c r="C27" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27">
-        <v>0</v>
-      </c>
-      <c r="E27" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <f>ROW()-2</f>
-        <v>26</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28" t="s">
+        <v>4</v>
+      </c>
+      <c r="F28" t="s">
+        <v>110</v>
+      </c>
+      <c r="G28" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <f t="shared" si="1"/>
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
         <v>90</v>
       </c>
-      <c r="C28" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28">
-        <v>0</v>
-      </c>
-      <c r="E28" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <f>ROW()-2</f>
-        <v>27</v>
-      </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29" t="s">
+        <v>4</v>
+      </c>
+      <c r="F29" t="s">
+        <v>109</v>
+      </c>
+      <c r="G29" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
         <v>91</v>
       </c>
-      <c r="C29" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29">
-        <v>0</v>
-      </c>
-      <c r="E29" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <f>ROW()-2</f>
-        <v>28</v>
-      </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>4</v>
+      </c>
+      <c r="F30" t="s">
+        <v>108</v>
+      </c>
+      <c r="G30" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
         <v>92</v>
       </c>
-      <c r="C30" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30">
-        <v>0</v>
-      </c>
-      <c r="E30" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <f>ROW()-2</f>
-        <v>29</v>
-      </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31" t="s">
+        <v>4</v>
+      </c>
+      <c r="F31" t="s">
+        <v>107</v>
+      </c>
+      <c r="G31" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
         <v>93</v>
       </c>
-      <c r="C31" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31">
-        <v>0</v>
-      </c>
-      <c r="E31" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <f>ROW()-2</f>
-        <v>30</v>
-      </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>4</v>
+      </c>
+      <c r="F32" t="s">
+        <v>106</v>
+      </c>
+      <c r="G32" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
         <v>94</v>
       </c>
-      <c r="C32" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32">
-        <v>0</v>
-      </c>
-      <c r="E32" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <f>ROW()-2</f>
-        <v>31</v>
-      </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" t="s">
+        <v>105</v>
+      </c>
+      <c r="G33" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <f t="shared" si="1"/>
+        <v>32</v>
+      </c>
+      <c r="B34" t="s">
         <v>95</v>
       </c>
-      <c r="C33" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33">
-        <v>0</v>
-      </c>
-      <c r="E33" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <f>ROW()-2</f>
-        <v>32</v>
-      </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" t="s">
+        <v>104</v>
+      </c>
+      <c r="G34" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
         <v>96</v>
       </c>
-      <c r="C34" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34">
-        <v>0</v>
-      </c>
-      <c r="E34" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <f>ROW()-2</f>
-        <v>33</v>
-      </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35" t="s">
+        <v>103</v>
+      </c>
+      <c r="G35" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
         <v>97</v>
       </c>
-      <c r="C35" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35">
-        <v>0</v>
-      </c>
-      <c r="E35" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <f>ROW()-2</f>
-        <v>34</v>
-      </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" t="s">
+        <v>102</v>
+      </c>
+      <c r="G36" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="B37" t="s">
         <v>98</v>
       </c>
-      <c r="C36" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36">
-        <v>0</v>
-      </c>
-      <c r="E36" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <f>ROW()-2</f>
-        <v>35</v>
-      </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
+        <v>6</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>4</v>
+      </c>
+      <c r="F37" t="s">
+        <v>101</v>
+      </c>
+      <c r="G37" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="B38" t="s">
         <v>99</v>
       </c>
-      <c r="C37" t="s">
-        <v>6</v>
-      </c>
-      <c r="D37">
-        <v>0</v>
-      </c>
-      <c r="E37" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <f>ROW()-2</f>
-        <v>36</v>
-      </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>4</v>
+      </c>
+      <c r="F38" t="s">
         <v>100</v>
       </c>
-      <c r="C38" t="s">
-        <v>6</v>
-      </c>
-      <c r="D38">
-        <v>0</v>
-      </c>
-      <c r="E38" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39">
-        <f t="shared" ref="A39:A45" si="1">ROW()-2</f>
+        <f t="shared" ref="A39:A45" si="2">ROW()-2</f>
         <v>37</v>
       </c>
       <c r="B39" t="s">
+        <v>70</v>
+      </c>
+      <c r="C39" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" t="s">
         <v>71</v>
       </c>
-      <c r="C39" t="s">
-        <v>6</v>
-      </c>
-      <c r="D39">
-        <v>0</v>
-      </c>
-      <c r="E39" t="s">
-        <v>4</v>
-      </c>
-      <c r="F39" t="s">
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <f t="shared" si="2"/>
+        <v>38</v>
+      </c>
+      <c r="B40" t="s">
+        <v>69</v>
+      </c>
+      <c r="C40" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40" t="s">
+        <v>4</v>
+      </c>
+      <c r="F40" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <f t="shared" si="1"/>
-        <v>38</v>
-      </c>
-      <c r="B40" t="s">
-        <v>70</v>
-      </c>
-      <c r="C40" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40">
-        <v>0</v>
-      </c>
-      <c r="E40" t="s">
-        <v>4</v>
-      </c>
-      <c r="F40" t="s">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <f t="shared" si="2"/>
+        <v>39</v>
+      </c>
+      <c r="B41" t="s">
+        <v>68</v>
+      </c>
+      <c r="C41" t="s">
+        <v>6</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>4</v>
+      </c>
+      <c r="F41" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="B42" t="s">
+        <v>67</v>
+      </c>
+      <c r="C42" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>4</v>
+      </c>
+      <c r="F42" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <f t="shared" si="1"/>
-        <v>39</v>
-      </c>
-      <c r="B41" t="s">
-        <v>69</v>
-      </c>
-      <c r="C41" t="s">
-        <v>6</v>
-      </c>
-      <c r="D41">
-        <v>0</v>
-      </c>
-      <c r="E41" t="s">
-        <v>4</v>
-      </c>
-      <c r="F41" t="s">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <f t="shared" si="2"/>
+        <v>41</v>
+      </c>
+      <c r="B43" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="B42" t="s">
-        <v>68</v>
-      </c>
-      <c r="C42" t="s">
-        <v>6</v>
-      </c>
-      <c r="D42">
-        <v>0</v>
-      </c>
-      <c r="E42" t="s">
-        <v>4</v>
-      </c>
-      <c r="F42" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <f t="shared" si="1"/>
-        <v>41</v>
-      </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43" t="s">
+        <v>4</v>
+      </c>
+      <c r="F43" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <f t="shared" si="2"/>
+        <v>42</v>
+      </c>
+      <c r="B44" t="s">
         <v>76</v>
       </c>
-      <c r="C43" t="s">
-        <v>6</v>
-      </c>
-      <c r="D43">
-        <v>0</v>
-      </c>
-      <c r="E43" t="s">
-        <v>4</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="C44" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44" t="s">
+        <v>4</v>
+      </c>
+      <c r="F44" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <f t="shared" si="2"/>
+        <v>43</v>
+      </c>
+      <c r="B45" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <f t="shared" si="1"/>
-        <v>42</v>
-      </c>
-      <c r="B44" t="s">
-        <v>77</v>
-      </c>
-      <c r="C44" t="s">
-        <v>6</v>
-      </c>
-      <c r="D44">
-        <v>0</v>
-      </c>
-      <c r="E44" t="s">
-        <v>4</v>
-      </c>
-      <c r="F44" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <f t="shared" si="1"/>
-        <v>43</v>
-      </c>
-      <c r="B45" t="s">
-        <v>80</v>
-      </c>
       <c r="C45" t="s">
         <v>6</v>
       </c>
@@ -1633,16 +1837,16 @@
         <v>4</v>
       </c>
       <c r="F45" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46">
         <f>ROW()-2</f>
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C46" t="s">
         <v>6</v>
@@ -1654,7 +1858,7 @@
         <v>4</v>
       </c>
       <c r="F46" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated CardValue excel sheet to include the card combinations
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shawn\Downloads\UNR\CS 425\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CB73AB4-0E8D-45CF-818B-559F3FD426F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9772D775-6C90-4D95-A67E-8415107ABC32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4305" yWindow="1035" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CardValue" sheetId="1" r:id="rId1"/>
@@ -798,16 +798,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G46"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="24.88671875" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" customWidth="1"/>
-    <col min="6" max="6" width="101.6640625" customWidth="1"/>
-    <col min="7" max="7" width="121.44140625" customWidth="1"/>
+    <col min="2" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="101.7109375" customWidth="1"/>
+    <col min="7" max="7" width="121.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -830,7 +830,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>ROW()-2</f>
         <v>0</v>
@@ -854,7 +854,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" ref="A3:A21" si="0">ROW()-2</f>
         <v>1</v>
@@ -878,7 +878,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -902,7 +902,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -926,7 +926,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -950,7 +950,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -974,7 +974,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -998,7 +998,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1022,7 +1022,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1046,7 +1046,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1070,7 +1070,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1094,7 +1094,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1118,7 +1118,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1142,7 +1142,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1166,7 +1166,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1190,7 +1190,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1214,7 +1214,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1238,7 +1238,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1262,7 +1262,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1286,7 +1286,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1310,7 +1310,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" ref="A22:A38" si="1">ROW()-2</f>
         <v>20</v>
@@ -1334,7 +1334,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="1"/>
         <v>21</v>
@@ -1358,7 +1358,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="1"/>
         <v>22</v>
@@ -1382,7 +1382,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="1"/>
         <v>23</v>
@@ -1406,7 +1406,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="1"/>
         <v>24</v>
@@ -1430,7 +1430,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
         <f t="shared" si="1"/>
         <v>25</v>
@@ -1454,7 +1454,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
         <f t="shared" si="1"/>
         <v>26</v>
@@ -1478,7 +1478,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
         <f t="shared" si="1"/>
         <v>27</v>
@@ -1502,7 +1502,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
         <f t="shared" si="1"/>
         <v>28</v>
@@ -1526,7 +1526,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
         <f t="shared" si="1"/>
         <v>29</v>
@@ -1550,7 +1550,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
         <f t="shared" si="1"/>
         <v>30</v>
@@ -1574,7 +1574,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33">
         <f t="shared" si="1"/>
         <v>31</v>
@@ -1598,7 +1598,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34">
         <f t="shared" si="1"/>
         <v>32</v>
@@ -1622,7 +1622,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35">
         <f t="shared" si="1"/>
         <v>33</v>
@@ -1646,7 +1646,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36">
         <f t="shared" si="1"/>
         <v>34</v>
@@ -1670,7 +1670,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37">
         <f t="shared" si="1"/>
         <v>35</v>
@@ -1694,7 +1694,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38">
         <f t="shared" si="1"/>
         <v>36</v>
@@ -1718,7 +1718,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39">
         <f t="shared" ref="A39:A45" si="2">ROW()-2</f>
         <v>37</v>
@@ -1739,7 +1739,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40">
         <f t="shared" si="2"/>
         <v>38</v>
@@ -1760,7 +1760,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41">
         <f t="shared" si="2"/>
         <v>39</v>
@@ -1781,7 +1781,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42">
         <f t="shared" si="2"/>
         <v>40</v>
@@ -1802,7 +1802,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43">
         <f t="shared" si="2"/>
         <v>41</v>
@@ -1823,7 +1823,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44">
         <f t="shared" si="2"/>
         <v>42</v>
@@ -1844,7 +1844,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45">
         <f t="shared" si="2"/>
         <v>43</v>
@@ -1865,7 +1865,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46">
         <f>ROW()-2</f>
         <v>44</v>
@@ -1894,13 +1894,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F568835D-C5E1-4D14-A337-01CA5B66900E}">
   <dimension ref="A1:H46"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="26.109375" customWidth="1"/>
-    <col min="8" max="8" width="21.88671875" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" customWidth="1"/>
+    <col min="5" max="5" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>135</v>
       </c>
@@ -1926,7 +1927,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1955,16 +1956,16 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="str">
         <f>VLOOKUP(B3, CardValue!A:B, 2, FALSE)</f>
-        <v>Syringe</v>
+        <v>Bandage</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1977,14 +1978,14 @@
         <v>0.1</v>
       </c>
       <c r="G3">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H3" t="str">
         <f>VLOOKUP(G3, CardValue!A:B, 2, FALSE)</f>
-        <v>Antidote Potion</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Adrenal Medkit</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1996,24 +1997,24 @@
         <v>Bandage</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E4" t="str">
         <f>VLOOKUP(D4, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Pills</v>
       </c>
       <c r="F4">
         <v>0.1</v>
       </c>
       <c r="G4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H4" t="str">
         <f>VLOOKUP(G4, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Combat Patch</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2025,24 +2026,24 @@
         <v>Bandage</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E5" t="str">
         <f>VLOOKUP(D5, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Rage Pill</v>
       </c>
       <c r="F5">
         <v>0.1</v>
       </c>
       <c r="G5">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H5" t="str">
         <f>VLOOKUP(G5, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Berserker Wrap</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2054,24 +2055,24 @@
         <v>Bandage</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E6" t="str">
         <f>VLOOKUP(D6, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Drugs</v>
       </c>
       <c r="F6">
         <v>0.1</v>
       </c>
       <c r="G6">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H6" t="str">
         <f>VLOOKUP(G6, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Stimulant Wrap</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2083,33 +2084,33 @@
         <v>Bandage</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E7" t="str">
         <f>VLOOKUP(D7, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Beer</v>
       </c>
       <c r="F7">
         <v>0.1</v>
       </c>
       <c r="G7">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H7" t="str">
         <f>VLOOKUP(G7, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Liquid Courage Kit</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" t="str">
         <f>VLOOKUP(B8, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Syringe</v>
       </c>
       <c r="D8">
         <v>2</v>
@@ -2122,139 +2123,139 @@
         <v>0.1</v>
       </c>
       <c r="G8">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H8" t="str">
         <f>VLOOKUP(G8, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Rapid Recovery Injector</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" t="str">
         <f>VLOOKUP(B9, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Syringe</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" t="str">
         <f>VLOOKUP(D9, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Revival Serum</v>
       </c>
       <c r="F9">
         <v>0.1</v>
       </c>
       <c r="G9">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="H9" t="str">
         <f>VLOOKUP(G9, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Phoenix Shot</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="str">
         <f>VLOOKUP(B10, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Syringe</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E10" t="str">
         <f>VLOOKUP(D10, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Beer</v>
       </c>
       <c r="F10">
         <v>0.1</v>
       </c>
       <c r="G10">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="H10" t="str">
         <f>VLOOKUP(G10, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Boosted Buzz</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C11" t="str">
         <f>VLOOKUP(B11, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Pills</v>
       </c>
       <c r="D11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E11" t="str">
         <f>VLOOKUP(D11, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Rage Pill</v>
       </c>
       <c r="F11">
         <v>0.1</v>
       </c>
       <c r="G11">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="H11" t="str">
         <f>VLOOKUP(G11, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Overdrive Dose</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C12" t="str">
         <f>VLOOKUP(B12, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Pills</v>
       </c>
       <c r="D12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" t="str">
         <f>VLOOKUP(D12, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Syringe</v>
       </c>
       <c r="F12">
         <v>0.1</v>
       </c>
       <c r="G12">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="H12" t="str">
         <f>VLOOKUP(G12, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Combat Stimulant</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C13" t="str">
         <f>VLOOKUP(B13, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Pills</v>
       </c>
       <c r="D13">
         <v>2</v>
@@ -2267,139 +2268,139 @@
         <v>0.1</v>
       </c>
       <c r="G13">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="H13" t="str">
         <f>VLOOKUP(G13, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Balanced Formula</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C14" t="str">
         <f>VLOOKUP(B14, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Pills</v>
       </c>
       <c r="D14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" t="str">
         <f>VLOOKUP(D14, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Revival Serum</v>
       </c>
       <c r="F14">
         <v>0.1</v>
       </c>
       <c r="G14">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="H14" t="str">
         <f>VLOOKUP(G14, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Rebirth Capsule</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C15" t="str">
         <f>VLOOKUP(B15, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Pills</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E15" t="str">
         <f>VLOOKUP(D15, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Drugs</v>
       </c>
       <c r="F15">
         <v>0.1</v>
       </c>
       <c r="G15">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H15" t="str">
         <f>VLOOKUP(G15, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Titan Formula</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C16" t="str">
         <f>VLOOKUP(B16, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Pills</v>
       </c>
       <c r="D16">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E16" t="str">
         <f>VLOOKUP(D16, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Beer</v>
       </c>
       <c r="F16">
         <v>0.1</v>
       </c>
       <c r="G16">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="H16" t="str">
         <f>VLOOKUP(G16, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Battle Brew</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C17" t="str">
         <f>VLOOKUP(B17, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Rage Pill</v>
       </c>
       <c r="D17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="str">
         <f>VLOOKUP(D17, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Syringe</v>
       </c>
       <c r="F17">
         <v>0.1</v>
       </c>
       <c r="G17">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="H17" t="str">
         <f>VLOOKUP(G17, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Adrenal Surge</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C18" t="str">
         <f>VLOOKUP(B18, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Rage Pill</v>
       </c>
       <c r="D18">
         <v>2</v>
@@ -2412,110 +2413,110 @@
         <v>0.1</v>
       </c>
       <c r="G18">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="H18" t="str">
         <f>VLOOKUP(G18, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Berserker Serum</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C19" t="str">
         <f>VLOOKUP(B19, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Rage Pill</v>
       </c>
       <c r="D19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E19" t="str">
         <f>VLOOKUP(D19, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Revival Serum</v>
       </c>
       <c r="F19">
         <v>0.1</v>
       </c>
       <c r="G19">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="H19" t="str">
         <f>VLOOKUP(G19, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Fury Rebirth</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C20" t="str">
         <f>VLOOKUP(B20, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Rage Pill</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E20" t="str">
         <f>VLOOKUP(D20, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Drugs</v>
       </c>
       <c r="F20">
         <v>0.1</v>
       </c>
       <c r="G20">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="H20" t="str">
         <f>VLOOKUP(G20, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Aggression Compound</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C21" t="str">
         <f>VLOOKUP(B21, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Rage Pill</v>
       </c>
       <c r="D21">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E21" t="str">
         <f>VLOOKUP(D21, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Beer</v>
       </c>
       <c r="F21">
         <v>0.1</v>
       </c>
       <c r="G21">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="H21" t="str">
         <f>VLOOKUP(G21, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Drunken Rage</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C22" t="str">
         <f>VLOOKUP(B22, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Drugs</v>
       </c>
       <c r="D22">
         <v>2</v>
@@ -2528,159 +2529,159 @@
         <v>0.1</v>
       </c>
       <c r="G22">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="H22" t="str">
         <f>VLOOKUP(G22, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Adrenal Mix</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C23" t="str">
         <f>VLOOKUP(B23, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Drugs</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" t="str">
         <f>VLOOKUP(D23, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Syringe</v>
       </c>
       <c r="F23">
         <v>0.1</v>
       </c>
       <c r="G23">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="H23" t="str">
         <f>VLOOKUP(G23, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Reflex Booster</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C24" t="str">
         <f>VLOOKUP(B24, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Drugs</v>
       </c>
       <c r="D24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E24" t="str">
         <f>VLOOKUP(D24, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Revival Serum</v>
       </c>
       <c r="F24">
         <v>0.1</v>
       </c>
       <c r="G24">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="H24" t="str">
         <f>VLOOKUP(G24, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Bio-Regen Formula</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>23</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C25" t="str">
         <f>VLOOKUP(B25, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Drugs</v>
       </c>
       <c r="D25">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E25" t="str">
         <f>VLOOKUP(D25, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Beer</v>
       </c>
       <c r="F25">
         <v>0.1</v>
       </c>
       <c r="G25">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="H25" t="str">
         <f>VLOOKUP(G25, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Nerve Enhancer</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C26" t="str">
         <f>VLOOKUP(B26, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Medkit</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E26" t="str">
         <f>VLOOKUP(D26, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Beer</v>
       </c>
       <c r="F26">
         <v>0.1</v>
       </c>
       <c r="G26">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="H26" t="str">
         <f>VLOOKUP(G26, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Survivor's Brew</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>25</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C27" t="str">
         <f>VLOOKUP(B27, CardValue!A:B, 2, FALSE)</f>
-        <v>Bandage</v>
+        <v>Beer</v>
       </c>
       <c r="D27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27" t="str">
         <f>VLOOKUP(D27, CardValue!A:B, 2, FALSE)</f>
-        <v>Medkit</v>
+        <v>Revival Serum</v>
       </c>
       <c r="F27">
         <v>0.1</v>
       </c>
       <c r="G27">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="H27" t="str">
         <f>VLOOKUP(G27, CardValue!A:B, 2, FALSE)</f>
-        <v>Field Surgery Kit</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Soul Brew</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>26</v>
       </c>
@@ -2709,7 +2710,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>27</v>
       </c>
@@ -2738,7 +2739,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>28</v>
       </c>
@@ -2767,7 +2768,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>29</v>
       </c>
@@ -2796,7 +2797,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>30</v>
       </c>
@@ -2825,7 +2826,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>31</v>
       </c>
@@ -2854,7 +2855,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>32</v>
       </c>
@@ -2883,7 +2884,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>33</v>
       </c>
@@ -2912,7 +2913,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>34</v>
       </c>
@@ -2941,7 +2942,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>35</v>
       </c>
@@ -2970,7 +2971,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>36</v>
       </c>
@@ -2999,7 +3000,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>37</v>
       </c>
@@ -3028,7 +3029,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>38</v>
       </c>
@@ -3057,7 +3058,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>39</v>
       </c>
@@ -3086,7 +3087,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>40</v>
       </c>
@@ -3115,7 +3116,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>41</v>
       </c>
@@ -3144,7 +3145,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>42</v>
       </c>
@@ -3173,7 +3174,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>43</v>
       </c>
@@ -3202,7 +3203,7 @@
         <v>Field Surgery Kit</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>44</v>
       </c>

</xml_diff>

<commit_message>
changed some of the names of the items since professor didn't like them
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9772D775-6C90-4D95-A67E-8415107ABC32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{739956DE-BC89-40EB-B22D-D12A4A5AC757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4305" yWindow="1035" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4305" yWindow="1035" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CardValue" sheetId="1" r:id="rId1"/>
@@ -98,27 +98,15 @@
     <t xml:space="preserve"> Automatically revives the player if the player reaches 0 health (only once) (10% - 20%)</t>
   </si>
   <si>
-    <t>Pills</t>
-  </si>
-  <si>
     <t xml:space="preserve"> increases attack (20% - 25%)</t>
   </si>
   <si>
-    <t>Rage Pill</t>
-  </si>
-  <si>
     <t xml:space="preserve"> increases attack (20% - 25%) but also decreases defense and health (10% - 15%)</t>
   </si>
   <si>
-    <t>Drugs</t>
-  </si>
-  <si>
     <t xml:space="preserve"> increases defense and attack (20% - 25%)</t>
   </si>
   <si>
-    <t>Beer</t>
-  </si>
-  <si>
     <t xml:space="preserve"> increases player’s critical chance (15% - 25%) (allows the player to deal increased damage)</t>
   </si>
   <si>
@@ -170,9 +158,6 @@
     <t xml:space="preserve"> increases critical damage by (Syringe % + (rarity of card)) for 3 turns and revives player to (Revival Serum % + (rarity of card))</t>
   </si>
   <si>
-    <t>Boosted Buzz</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Increases critical damage by (Syringe % + (rarity of card)) and increases critical chance by (Beer % + (rarity of card)) for 2 turns</t>
   </si>
   <si>
@@ -332,9 +317,6 @@
     <t>Aggression Compound</t>
   </si>
   <si>
-    <t>Drunken Rage</t>
-  </si>
-  <si>
     <t>Adrenal Mix</t>
   </si>
   <si>
@@ -480,6 +462,24 @@
   </si>
   <si>
     <t>Result Card Name(Not involved in script)</t>
+  </si>
+  <si>
+    <t>Stamina Capsule</t>
+  </si>
+  <si>
+    <t>Reflex Tonic</t>
+  </si>
+  <si>
+    <t>Battle Frenzy</t>
+  </si>
+  <si>
+    <t>Fury Catalyst</t>
+  </si>
+  <si>
+    <t>Emergency Capsule</t>
+  </si>
+  <si>
+    <t>Enhanced Focus</t>
   </si>
 </sst>
 </file>
@@ -827,7 +827,7 @@
         <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -851,7 +851,7 @@
         <v>8</v>
       </c>
       <c r="G2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -875,7 +875,7 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -899,7 +899,7 @@
         <v>12</v>
       </c>
       <c r="G4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -923,7 +923,7 @@
         <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -932,22 +932,22 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F6" t="s">
-        <v>16</v>
-      </c>
       <c r="G6" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -956,7 +956,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>140</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -968,19 +968,19 @@
         <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
-        <f t="shared" si="0"/>
+        <f>ROW()-2</f>
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>137</v>
       </c>
       <c r="C8" t="s">
         <v>6</v>
@@ -992,10 +992,10 @@
         <v>4</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1004,7 +1004,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>138</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
@@ -1016,10 +1016,10 @@
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1028,7 +1028,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
@@ -1040,10 +1040,10 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G10" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1052,7 +1052,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
@@ -1064,10 +1064,10 @@
         <v>4</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G11" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1076,7 +1076,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C12" t="s">
         <v>6</v>
@@ -1088,10 +1088,10 @@
         <v>4</v>
       </c>
       <c r="F12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1100,7 +1100,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
         <v>6</v>
@@ -1112,10 +1112,10 @@
         <v>4</v>
       </c>
       <c r="F13" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G13" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1124,7 +1124,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C14" t="s">
         <v>6</v>
@@ -1136,10 +1136,10 @@
         <v>4</v>
       </c>
       <c r="F14" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G14" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1148,7 +1148,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C15" t="s">
         <v>6</v>
@@ -1160,10 +1160,10 @@
         <v>4</v>
       </c>
       <c r="F15" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1172,7 +1172,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
         <v>6</v>
@@ -1184,10 +1184,10 @@
         <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G16" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1196,7 +1196,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
         <v>6</v>
@@ -1208,10 +1208,10 @@
         <v>4</v>
       </c>
       <c r="F17" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="G17" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1220,7 +1220,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C18" t="s">
         <v>6</v>
@@ -1232,10 +1232,10 @@
         <v>4</v>
       </c>
       <c r="F18" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1244,7 +1244,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C19" t="s">
         <v>6</v>
@@ -1256,10 +1256,10 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G19" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1268,7 +1268,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
         <v>6</v>
@@ -1280,10 +1280,10 @@
         <v>4</v>
       </c>
       <c r="F20" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G20" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1292,7 +1292,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>142</v>
       </c>
       <c r="C21" t="s">
         <v>6</v>
@@ -1304,10 +1304,10 @@
         <v>4</v>
       </c>
       <c r="F21" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G21" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1316,7 +1316,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C22" t="s">
         <v>6</v>
@@ -1328,10 +1328,10 @@
         <v>4</v>
       </c>
       <c r="F22" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="G22" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1340,7 +1340,7 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C23" t="s">
         <v>6</v>
@@ -1352,10 +1352,10 @@
         <v>4</v>
       </c>
       <c r="F23" t="s">
+        <v>109</v>
+      </c>
+      <c r="G23" t="s">
         <v>115</v>
-      </c>
-      <c r="G23" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1364,7 +1364,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C24" t="s">
         <v>6</v>
@@ -1376,10 +1376,10 @@
         <v>4</v>
       </c>
       <c r="F24" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="G24" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1388,7 +1388,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
         <v>6</v>
@@ -1400,10 +1400,10 @@
         <v>4</v>
       </c>
       <c r="F25" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="G25" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1412,7 +1412,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C26" t="s">
         <v>6</v>
@@ -1424,10 +1424,10 @@
         <v>4</v>
       </c>
       <c r="F26" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="G26" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1436,7 +1436,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C27" t="s">
         <v>6</v>
@@ -1448,10 +1448,10 @@
         <v>4</v>
       </c>
       <c r="F27" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="G27" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1460,7 +1460,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C28" t="s">
         <v>6</v>
@@ -1472,10 +1472,10 @@
         <v>4</v>
       </c>
       <c r="F28" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="G28" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1484,7 +1484,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C29" t="s">
         <v>6</v>
@@ -1496,10 +1496,10 @@
         <v>4</v>
       </c>
       <c r="F29" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G29" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1508,7 +1508,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C30" t="s">
         <v>6</v>
@@ -1520,10 +1520,10 @@
         <v>4</v>
       </c>
       <c r="F30" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G30" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1532,7 +1532,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C31" t="s">
         <v>6</v>
@@ -1544,10 +1544,10 @@
         <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G31" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1556,7 +1556,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>139</v>
       </c>
       <c r="C32" t="s">
         <v>6</v>
@@ -1568,10 +1568,10 @@
         <v>4</v>
       </c>
       <c r="F32" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="G32" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -1580,7 +1580,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
         <v>6</v>
@@ -1592,10 +1592,10 @@
         <v>4</v>
       </c>
       <c r="F33" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="G33" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -1604,7 +1604,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C34" t="s">
         <v>6</v>
@@ -1616,10 +1616,10 @@
         <v>4</v>
       </c>
       <c r="F34" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="G34" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -1628,7 +1628,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C35" t="s">
         <v>6</v>
@@ -1640,10 +1640,10 @@
         <v>4</v>
       </c>
       <c r="F35" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="G35" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -1652,7 +1652,7 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C36" t="s">
         <v>6</v>
@@ -1664,10 +1664,10 @@
         <v>4</v>
       </c>
       <c r="F36" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G36" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -1676,7 +1676,7 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C37" t="s">
         <v>6</v>
@@ -1688,10 +1688,10 @@
         <v>4</v>
       </c>
       <c r="F37" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="G37" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -1700,7 +1700,7 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C38" t="s">
         <v>6</v>
@@ -1712,10 +1712,10 @@
         <v>4</v>
       </c>
       <c r="F38" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G38" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -1724,7 +1724,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C39" t="s">
         <v>6</v>
@@ -1736,7 +1736,7 @@
         <v>4</v>
       </c>
       <c r="F39" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -1745,7 +1745,7 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C40" t="s">
         <v>6</v>
@@ -1757,7 +1757,7 @@
         <v>4</v>
       </c>
       <c r="F40" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -1766,7 +1766,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C41" t="s">
         <v>6</v>
@@ -1778,7 +1778,7 @@
         <v>4</v>
       </c>
       <c r="F41" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -1787,7 +1787,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C42" t="s">
         <v>6</v>
@@ -1799,7 +1799,7 @@
         <v>4</v>
       </c>
       <c r="F42" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -1808,7 +1808,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C43" t="s">
         <v>6</v>
@@ -1820,7 +1820,7 @@
         <v>4</v>
       </c>
       <c r="F43" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -1829,7 +1829,7 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C44" t="s">
         <v>6</v>
@@ -1841,7 +1841,7 @@
         <v>4</v>
       </c>
       <c r="F44" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -1850,7 +1850,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C45" t="s">
         <v>6</v>
@@ -1862,7 +1862,7 @@
         <v>4</v>
       </c>
       <c r="F45" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -1871,7 +1871,7 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C46" t="s">
         <v>6</v>
@@ -1883,7 +1883,7 @@
         <v>4</v>
       </c>
       <c r="F46" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1903,28 +1903,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E1" t="s">
+        <v>133</v>
+      </c>
+      <c r="F1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G1" t="s">
         <v>135</v>
       </c>
-      <c r="B1" t="s">
+      <c r="H1" t="s">
         <v>136</v>
-      </c>
-      <c r="C1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D1" t="s">
-        <v>138</v>
-      </c>
-      <c r="E1" t="s">
-        <v>139</v>
-      </c>
-      <c r="F1" t="s">
-        <v>140</v>
-      </c>
-      <c r="G1" t="s">
-        <v>141</v>
-      </c>
-      <c r="H1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="E4" t="str">
         <f>VLOOKUP(D4, CardValue!A:B, 2, FALSE)</f>
-        <v>Pills</v>
+        <v>Emergency Capsule</v>
       </c>
       <c r="F4">
         <v>0.1</v>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="E5" t="str">
         <f>VLOOKUP(D5, CardValue!A:B, 2, FALSE)</f>
-        <v>Rage Pill</v>
+        <v>Fury Catalyst</v>
       </c>
       <c r="F5">
         <v>0.1</v>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="E6" t="str">
         <f>VLOOKUP(D6, CardValue!A:B, 2, FALSE)</f>
-        <v>Drugs</v>
+        <v>Stamina Capsule</v>
       </c>
       <c r="F6">
         <v>0.1</v>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="E7" t="str">
         <f>VLOOKUP(D7, CardValue!A:B, 2, FALSE)</f>
-        <v>Beer</v>
+        <v>Reflex Tonic</v>
       </c>
       <c r="F7">
         <v>0.1</v>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="E10" t="str">
         <f>VLOOKUP(D10, CardValue!A:B, 2, FALSE)</f>
-        <v>Beer</v>
+        <v>Reflex Tonic</v>
       </c>
       <c r="F10">
         <v>0.1</v>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="H10" t="str">
         <f>VLOOKUP(G10, CardValue!A:B, 2, FALSE)</f>
-        <v>Boosted Buzz</v>
+        <v>Enhanced Focus</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -2197,14 +2197,14 @@
       </c>
       <c r="C11" t="str">
         <f>VLOOKUP(B11, CardValue!A:B, 2, FALSE)</f>
-        <v>Pills</v>
+        <v>Emergency Capsule</v>
       </c>
       <c r="D11">
         <v>5</v>
       </c>
       <c r="E11" t="str">
         <f>VLOOKUP(D11, CardValue!A:B, 2, FALSE)</f>
-        <v>Rage Pill</v>
+        <v>Fury Catalyst</v>
       </c>
       <c r="F11">
         <v>0.1</v>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="C12" t="str">
         <f>VLOOKUP(B12, CardValue!A:B, 2, FALSE)</f>
-        <v>Pills</v>
+        <v>Emergency Capsule</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="C13" t="str">
         <f>VLOOKUP(B13, CardValue!A:B, 2, FALSE)</f>
-        <v>Pills</v>
+        <v>Emergency Capsule</v>
       </c>
       <c r="D13">
         <v>2</v>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="C14" t="str">
         <f>VLOOKUP(B14, CardValue!A:B, 2, FALSE)</f>
-        <v>Pills</v>
+        <v>Emergency Capsule</v>
       </c>
       <c r="D14">
         <v>3</v>
@@ -2313,14 +2313,14 @@
       </c>
       <c r="C15" t="str">
         <f>VLOOKUP(B15, CardValue!A:B, 2, FALSE)</f>
-        <v>Pills</v>
+        <v>Emergency Capsule</v>
       </c>
       <c r="D15">
         <v>6</v>
       </c>
       <c r="E15" t="str">
         <f>VLOOKUP(D15, CardValue!A:B, 2, FALSE)</f>
-        <v>Drugs</v>
+        <v>Stamina Capsule</v>
       </c>
       <c r="F15">
         <v>0.1</v>
@@ -2342,14 +2342,14 @@
       </c>
       <c r="C16" t="str">
         <f>VLOOKUP(B16, CardValue!A:B, 2, FALSE)</f>
-        <v>Pills</v>
+        <v>Emergency Capsule</v>
       </c>
       <c r="D16">
         <v>7</v>
       </c>
       <c r="E16" t="str">
         <f>VLOOKUP(D16, CardValue!A:B, 2, FALSE)</f>
-        <v>Beer</v>
+        <v>Reflex Tonic</v>
       </c>
       <c r="F16">
         <v>0.1</v>
@@ -2371,7 +2371,7 @@
       </c>
       <c r="C17" t="str">
         <f>VLOOKUP(B17, CardValue!A:B, 2, FALSE)</f>
-        <v>Rage Pill</v>
+        <v>Fury Catalyst</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="C18" t="str">
         <f>VLOOKUP(B18, CardValue!A:B, 2, FALSE)</f>
-        <v>Rage Pill</v>
+        <v>Fury Catalyst</v>
       </c>
       <c r="D18">
         <v>2</v>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="C19" t="str">
         <f>VLOOKUP(B19, CardValue!A:B, 2, FALSE)</f>
-        <v>Rage Pill</v>
+        <v>Fury Catalyst</v>
       </c>
       <c r="D19">
         <v>3</v>
@@ -2458,14 +2458,14 @@
       </c>
       <c r="C20" t="str">
         <f>VLOOKUP(B20, CardValue!A:B, 2, FALSE)</f>
-        <v>Rage Pill</v>
+        <v>Fury Catalyst</v>
       </c>
       <c r="D20">
         <v>6</v>
       </c>
       <c r="E20" t="str">
         <f>VLOOKUP(D20, CardValue!A:B, 2, FALSE)</f>
-        <v>Drugs</v>
+        <v>Stamina Capsule</v>
       </c>
       <c r="F20">
         <v>0.1</v>
@@ -2487,14 +2487,14 @@
       </c>
       <c r="C21" t="str">
         <f>VLOOKUP(B21, CardValue!A:B, 2, FALSE)</f>
-        <v>Rage Pill</v>
+        <v>Fury Catalyst</v>
       </c>
       <c r="D21">
         <v>7</v>
       </c>
       <c r="E21" t="str">
         <f>VLOOKUP(D21, CardValue!A:B, 2, FALSE)</f>
-        <v>Beer</v>
+        <v>Reflex Tonic</v>
       </c>
       <c r="F21">
         <v>0.1</v>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="H21" t="str">
         <f>VLOOKUP(G21, CardValue!A:B, 2, FALSE)</f>
-        <v>Drunken Rage</v>
+        <v>Battle Frenzy</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="C22" t="str">
         <f>VLOOKUP(B22, CardValue!A:B, 2, FALSE)</f>
-        <v>Drugs</v>
+        <v>Stamina Capsule</v>
       </c>
       <c r="D22">
         <v>2</v>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="C23" t="str">
         <f>VLOOKUP(B23, CardValue!A:B, 2, FALSE)</f>
-        <v>Drugs</v>
+        <v>Stamina Capsule</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="C24" t="str">
         <f>VLOOKUP(B24, CardValue!A:B, 2, FALSE)</f>
-        <v>Drugs</v>
+        <v>Stamina Capsule</v>
       </c>
       <c r="D24">
         <v>3</v>
@@ -2603,14 +2603,14 @@
       </c>
       <c r="C25" t="str">
         <f>VLOOKUP(B25, CardValue!A:B, 2, FALSE)</f>
-        <v>Drugs</v>
+        <v>Stamina Capsule</v>
       </c>
       <c r="D25">
         <v>7</v>
       </c>
       <c r="E25" t="str">
         <f>VLOOKUP(D25, CardValue!A:B, 2, FALSE)</f>
-        <v>Beer</v>
+        <v>Reflex Tonic</v>
       </c>
       <c r="F25">
         <v>0.1</v>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="E26" t="str">
         <f>VLOOKUP(D26, CardValue!A:B, 2, FALSE)</f>
-        <v>Beer</v>
+        <v>Reflex Tonic</v>
       </c>
       <c r="F26">
         <v>0.1</v>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="C27" t="str">
         <f>VLOOKUP(B27, CardValue!A:B, 2, FALSE)</f>
-        <v>Beer</v>
+        <v>Reflex Tonic</v>
       </c>
       <c r="D27">
         <v>3</v>

</xml_diff>

<commit_message>
updated interactables, visuals and battle game over. most of everything resets when battle starts over, but card does not reset
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shawn\Downloads\UNR\CS 425\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C198D777-9143-4671-A8F1-BDBAE6743156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73569458-9B7A-4E32-BFA4-BCA4188080E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7188" yWindow="5940" windowWidth="15852" windowHeight="7524" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="30960" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CardValue" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="55">
   <si>
     <t>ID</t>
   </si>
@@ -152,9 +152,6 @@
     <t>Brugs</t>
   </si>
   <si>
-    <t>Increases Attack 10</t>
-  </si>
-  <si>
     <t>Heals player (15%)</t>
   </si>
   <si>
@@ -164,33 +161,18 @@
     <t>Heals a large amount of health (50%)</t>
   </si>
   <si>
-    <t>Increases Attack 20%</t>
-  </si>
-  <si>
-    <t>Increases attack ( 25%) but also decreases defense and health (5%)</t>
-  </si>
-  <si>
     <t>Increases defense and attack (25%)</t>
   </si>
   <si>
     <t>Increases player’s critical chance (20%)</t>
   </si>
   <si>
-    <t>Increases Attack 5 and then 5 %</t>
-  </si>
-  <si>
-    <t>Heals player (10%) and then 10</t>
-  </si>
-  <si>
     <t>Give All Enemy 10 Damage</t>
   </si>
   <si>
     <t>Restores 100 Health</t>
   </si>
   <si>
-    <t>Restores 100% Health</t>
-  </si>
-  <si>
     <t>Increases Attack 5 and Reduce Health 5</t>
   </si>
   <si>
@@ -200,12 +182,6 @@
     <t>Give 1 enemy 100 Damage</t>
   </si>
   <si>
-    <t>ReduceHealth 20% and Add Attack 20%</t>
-  </si>
-  <si>
-    <t>ReduceHealth 20% and Add Defense 20%</t>
-  </si>
-  <si>
     <t>Add Health 50% and Reduce Defense 20%</t>
   </si>
   <si>
@@ -219,6 +195,27 @@
   </si>
   <si>
     <t>Fury Catalyst</t>
+  </si>
+  <si>
+    <t>Reduce Health 20% and Add Attack 20%</t>
+  </si>
+  <si>
+    <t>Reduce Health 20% and Add Defense 20%</t>
+  </si>
+  <si>
+    <t>Increases Attack by 10</t>
+  </si>
+  <si>
+    <t>Increases Attack by 20%</t>
+  </si>
+  <si>
+    <t>Increases attack (25%) but also decreases defense and health (5%)</t>
+  </si>
+  <si>
+    <t>Increases Attack by 5 and then 5%</t>
+  </si>
+  <si>
+    <t>Restores 20 Health</t>
   </si>
 </sst>
 </file>
@@ -587,7 +584,7 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -608,7 +605,7 @@
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -629,7 +626,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -638,7 +635,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -650,7 +647,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -671,7 +668,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -692,7 +689,7 @@
         <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -713,7 +710,7 @@
         <v>4</v>
       </c>
       <c r="F8" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -734,7 +731,7 @@
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -755,7 +752,7 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -776,7 +773,7 @@
         <v>4</v>
       </c>
       <c r="F11" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -797,7 +794,7 @@
         <v>4</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -818,7 +815,7 @@
         <v>4</v>
       </c>
       <c r="F13" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -839,7 +836,7 @@
         <v>4</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -860,7 +857,7 @@
         <v>4</v>
       </c>
       <c r="F15" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -869,7 +866,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="C16" t="s">
         <v>6</v>
@@ -881,7 +878,7 @@
         <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -890,7 +887,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C17" t="s">
         <v>6</v>
@@ -902,7 +899,7 @@
         <v>4</v>
       </c>
       <c r="F17" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -923,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="F18" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -944,7 +941,7 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -965,7 +962,7 @@
         <v>4</v>
       </c>
       <c r="F20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -986,7 +983,7 @@
         <v>4</v>
       </c>
       <c r="F21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
improved alot of the UI to make it more visually appealing.
improved the UI to make it more visually appealing. (health bar in battle, turn update, and reward screen after successfully winning a battle)

inventory has some issue now where it won't close properly if opened at a different scene while the game is running.
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73569458-9B7A-4E32-BFA4-BCA4188080E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE13EE5-E8A7-479A-B75F-84A9F67A7AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="30960" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CardValue" sheetId="1" r:id="rId1"/>
@@ -149,9 +149,6 @@
     <t>Boosted Buzz</t>
   </si>
   <si>
-    <t>Brugs</t>
-  </si>
-  <si>
     <t>Heals player (15%)</t>
   </si>
   <si>
@@ -216,6 +213,9 @@
   </si>
   <si>
     <t>Restores 20 Health</t>
+  </si>
+  <si>
+    <t>Stamina Capsule</t>
   </si>
 </sst>
 </file>
@@ -584,7 +584,7 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -605,7 +605,7 @@
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -626,7 +626,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -635,7 +635,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -647,7 +647,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -668,7 +668,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -689,7 +689,7 @@
         <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -710,7 +710,7 @@
         <v>4</v>
       </c>
       <c r="F8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
@@ -731,7 +731,7 @@
         <v>4</v>
       </c>
       <c r="F9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -752,7 +752,7 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -773,7 +773,7 @@
         <v>4</v>
       </c>
       <c r="F11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -794,7 +794,7 @@
         <v>4</v>
       </c>
       <c r="F12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -815,7 +815,7 @@
         <v>4</v>
       </c>
       <c r="F13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -836,7 +836,7 @@
         <v>4</v>
       </c>
       <c r="F14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -857,7 +857,7 @@
         <v>4</v>
       </c>
       <c r="F15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -866,7 +866,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
         <v>6</v>
@@ -878,7 +878,7 @@
         <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -887,7 +887,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" t="s">
         <v>6</v>
@@ -899,7 +899,7 @@
         <v>4</v>
       </c>
       <c r="F17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -920,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="F18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -941,7 +941,7 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -962,7 +962,7 @@
         <v>4</v>
       </c>
       <c r="F20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -983,7 +983,7 @@
         <v>4</v>
       </c>
       <c r="F21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="E7" t="str">
         <f>VLOOKUP(D7, CardValue!A:B, 2, FALSE)</f>
-        <v>Brugs</v>
+        <v>Stamina Capsule</v>
       </c>
       <c r="F7">
         <v>0.1</v>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E10" t="str">
         <f>VLOOKUP(D10, CardValue!A:B, 2, FALSE)</f>
-        <v>Brugs</v>
+        <v>Stamina Capsule</v>
       </c>
       <c r="F10">
         <v>0.1</v>

</xml_diff>

<commit_message>
key interactable with door now works
also added a note in level_1 that guides player to find the key to unlock the door leading to the hospital
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE13EE5-E8A7-479A-B75F-84A9F67A7AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D56B3D0F-6FD8-4BE3-835A-B145348C0A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CardValue" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="57">
   <si>
     <t>ID</t>
   </si>
@@ -216,6 +216,12 @@
   </si>
   <si>
     <t>Stamina Capsule</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Use to unlock locked doors</t>
   </si>
 </sst>
 </file>
@@ -533,17 +539,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="7.77734375" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" customWidth="1"/>
+    <col min="2" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
     <col min="6" max="6" width="139" customWidth="1"/>
-    <col min="7" max="7" width="121.44140625" customWidth="1"/>
+    <col min="7" max="7" width="121.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -566,7 +572,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>ROW()-2</f>
         <v>0</v>
@@ -587,7 +593,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" ref="A3:A19" si="0">ROW()-2</f>
         <v>1</v>
@@ -608,7 +614,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -629,7 +635,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -650,7 +656,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -671,7 +677,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -692,7 +698,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <f>ROW()-2</f>
         <v>6</v>
@@ -713,7 +719,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -734,7 +740,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -755,7 +761,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -776,7 +782,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -797,7 +803,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -818,7 +824,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -839,7 +845,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -860,7 +866,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -881,7 +887,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -902,7 +908,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -923,7 +929,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -944,7 +950,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" ref="A20:A21" si="1">ROW()-2</f>
         <v>18</v>
@@ -965,9 +971,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
-        <f t="shared" si="1"/>
+        <f>ROW()-2</f>
         <v>19</v>
       </c>
       <c r="B21" t="s">
@@ -984,6 +990,27 @@
       </c>
       <c r="F21" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <f>ROW()-2</f>
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>4</v>
+      </c>
+      <c r="F22" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -994,14 +1021,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F568835D-C5E1-4D14-A337-01CA5B66900E}">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="26.109375" customWidth="1"/>
-    <col min="5" max="5" width="33.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.88671875" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" customWidth="1"/>
+    <col min="5" max="5" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -1027,7 +1054,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1056,7 +1083,7 @@
         <v>Liquid Courage Kit</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1085,7 +1112,7 @@
         <v>Medkit</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1114,7 +1141,7 @@
         <v>Phoenix Shot</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1143,7 +1170,7 @@
         <v>Emergency Capsule</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1172,7 +1199,7 @@
         <v>Fury Catalyst</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -1201,7 +1228,7 @@
         <v>Rapid Recovery Injector</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -1230,7 +1257,7 @@
         <v>Revival Serum</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -1259,7 +1286,7 @@
         <v>Stimulant Wrap</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1288,7 +1315,7 @@
         <v>Syringe</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1317,7 +1344,7 @@
         <v>Syringe</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
added an ending to the game
ending happens at level_2.
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D56B3D0F-6FD8-4BE3-835A-B145348C0A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B882353-C5F5-4198-846D-B26C24FFF1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="59">
   <si>
     <t>ID</t>
   </si>
@@ -222,6 +222,12 @@
   </si>
   <si>
     <t>Use to unlock locked doors</t>
+  </si>
+  <si>
+    <t>Cure</t>
+  </si>
+  <si>
+    <t>Use to cure someone of the zombie virus</t>
   </si>
 </sst>
 </file>
@@ -539,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="19.7109375" customWidth="1"/>
@@ -952,7 +958,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
-        <f t="shared" ref="A20:A21" si="1">ROW()-2</f>
+        <f t="shared" ref="A20" si="1">ROW()-2</f>
         <v>18</v>
       </c>
       <c r="B20" t="s">
@@ -1011,6 +1017,27 @@
       </c>
       <c r="F22" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <f>ROW() - 2</f>
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>4</v>
+      </c>
+      <c r="F23" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed music when pausing in battle, added more health interactables, and restarting from pause screen in battle now works
originally, the restart from the pause screen in battle only reset the player health. now it everything from when battle was first entered
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/CardValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B882353-C5F5-4198-846D-B26C24FFF1E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3040AA9-CC13-4E2E-AE88-30F7E2B8FD2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5370" yWindow="3555" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CardValue" sheetId="1" r:id="rId1"/>
@@ -206,9 +206,6 @@
     <t>Increases Attack by 20%</t>
   </si>
   <si>
-    <t>Increases attack (25%) but also decreases defense and health (5%)</t>
-  </si>
-  <si>
     <t>Increases Attack by 5 and then 5%</t>
   </si>
   <si>
@@ -228,6 +225,9 @@
   </si>
   <si>
     <t>Use to cure someone of the zombie virus</t>
+  </si>
+  <si>
+    <t>Increases attack (25%) but also decreases defense and health (50%)</t>
   </si>
 </sst>
 </file>
@@ -701,7 +701,7 @@
         <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -731,7 +731,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
@@ -827,7 +827,7 @@
         <v>4</v>
       </c>
       <c r="F13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -848,7 +848,7 @@
         <v>4</v>
       </c>
       <c r="F14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1004,19 +1004,19 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>4</v>
+      </c>
+      <c r="F22" t="s">
         <v>55</v>
-      </c>
-      <c r="C22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22" t="s">
-        <v>4</v>
-      </c>
-      <c r="F22" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1025,19 +1025,19 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>4</v>
+      </c>
+      <c r="F23" t="s">
         <v>57</v>
-      </c>
-      <c r="C23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23" t="s">
-        <v>4</v>
-      </c>
-      <c r="F23" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>